<commit_message>
Support simple 4-column wriggle input; auto-group into rings
- Sidebar: new inputs for points_per_ring (default 8) and prism_offset (default 0.038)
- prepare_wrs_data(): converts simple (POINT NO., E, N, Z) → full format
  by grouping rows into rings and filling RING NO., OFFSET, NUM. POINTS
- Auto-detect format: if NUM. POINTS column absent → use simple mode
- DTA: also reads first sheet (sheet_name=0) for flexibility
- Updated Sample_Wriggle_Survey_Input.xlsx: 4-column wriggle sheet + DTA sheet

https://claude.ai/code/session_01Dgd3MpcCstpJRMT2xbvcFn
</commit_message>
<xml_diff>
--- a/Sample_Wriggle_Survey_Input.xlsx
+++ b/Sample_Wriggle_Survey_Input.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Import Wriggle Data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Import Tunnel Axis (DTA)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Wriggle Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="DTA Data (Excel format)" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,13 +29,24 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C55A11"/>
       <sz val="10"/>
     </font>
     <font>
-      <b val="1"/>
+      <color rgb="00595959"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -49,7 +60,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00EBF3FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FAFAFA"/>
       </patternFill>
     </fill>
     <fill>
@@ -84,19 +100,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -463,416 +484,293 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>RING NO.</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>POINT NO.</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>EASTING (M.)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>NORTHING (M.)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ELEVATION (M.)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>OFFSET (M.)</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>NUM. POINTS</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>1</v>
+        <v>671704.6834</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>671704.6834</v>
+        <v>1507395.045</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>1507395.045</v>
-      </c>
-      <c r="E2" s="2" t="n">
         <v>-26.0029</v>
       </c>
-      <c r="F2" s="2" t="n">
-        <v>0.038</v>
-      </c>
-      <c r="G2" s="3" t="n">
-        <v>8</v>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>⚠️ Kural: Her ring için POINT NO. 1den baslar</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>2</v>
+        <v>671704.8665</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>671704.8665</v>
+        <v>1507394.862</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1507394.862</v>
-      </c>
-      <c r="E3" s="2" t="n">
         <v>-26.7536</v>
       </c>
-      <c r="F3" s="2" t="n">
-        <v>0.038</v>
-      </c>
-      <c r="G3" s="2" t="n"/>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Uygulama ring gruplarini otomatik hesaplar</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>3</v>
+        <v>671704.7862</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>671704.7862</v>
+        <v>1507394.957</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>1507394.957</v>
-      </c>
-      <c r="E4" s="2" t="n">
         <v>-27.527</v>
       </c>
-      <c r="F4" s="2" t="n">
-        <v>0.038</v>
-      </c>
-      <c r="G4" s="2" t="n"/>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Ring basina nokta sayisi sidebar da ayarlanir (orn. 8)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>4</v>
+        <v>671704.5866</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>671704.5866</v>
+        <v>1507395.171</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1507395.171</v>
-      </c>
-      <c r="E5" s="2" t="n">
         <v>-27.9933</v>
       </c>
-      <c r="F5" s="2" t="n">
-        <v>0.038</v>
-      </c>
-      <c r="G5" s="2" t="n"/>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Prizma offset sidebar da ayarlanir (orn. 0.038 m)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>5</v>
+        <v>671702.8676999999</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>671702.8676999999</v>
+        <v>1507396.971</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1507396.971</v>
-      </c>
-      <c r="E6" s="2" t="n">
         <v>-27.9951</v>
       </c>
-      <c r="F6" s="2" t="n">
-        <v>0.038</v>
-      </c>
-      <c r="G6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>6</v>
+        <v>671702.6382</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>671702.6382</v>
+        <v>1507397.203</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1507397.203</v>
-      </c>
-      <c r="E7" s="2" t="n">
         <v>-27.4416</v>
       </c>
-      <c r="F7" s="2" t="n">
-        <v>0.038</v>
-      </c>
-      <c r="G7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>7</v>
+        <v>671702.591</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>671702.591</v>
+        <v>1507397.244</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1507397.244</v>
-      </c>
-      <c r="E8" s="2" t="n">
         <v>-26.6604</v>
       </c>
-      <c r="F8" s="2" t="n">
-        <v>0.038</v>
-      </c>
-      <c r="G8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="B9" s="2" t="n">
+        <v>671702.8039000001</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>1507397.011</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>-25.9139</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>671705.5596</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>1507395.855</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>-26.0128</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>671705.7218000001</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>1507395.674</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>-26.746</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>671705.6372999999</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>1507395.767</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>-27.5342</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>671705.4195</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>1507395.991</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>-27.9994</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>671703.7396</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>1507397.789</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>-27.9921</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>671703.5187</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>1507398.033</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>-27.436</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>671703.4754999999</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>1507398.085</v>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>-26.6546</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="C9" s="2" t="n">
-        <v>671702.8039000001</v>
-      </c>
-      <c r="D9" s="2" t="n">
-        <v>1507397.011</v>
-      </c>
-      <c r="E9" s="2" t="n">
-        <v>-25.9139</v>
-      </c>
-      <c r="F9" s="2" t="n">
-        <v>0.038</v>
-      </c>
-      <c r="G9" s="2" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" s="2" t="n">
-        <v>671705.5596</v>
-      </c>
-      <c r="D10" s="2" t="n">
-        <v>1507395.855</v>
-      </c>
-      <c r="E10" s="2" t="n">
-        <v>-26.0128</v>
-      </c>
-      <c r="F10" s="2" t="n">
-        <v>0.038</v>
-      </c>
-      <c r="G10" s="3" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C11" s="2" t="n">
-        <v>671705.7218000001</v>
-      </c>
-      <c r="D11" s="2" t="n">
-        <v>1507395.674</v>
-      </c>
-      <c r="E11" s="2" t="n">
-        <v>-26.746</v>
-      </c>
-      <c r="F11" s="2" t="n">
-        <v>0.038</v>
-      </c>
-      <c r="G11" s="2" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C12" s="2" t="n">
-        <v>671705.6372999999</v>
-      </c>
-      <c r="D12" s="2" t="n">
-        <v>1507395.767</v>
-      </c>
-      <c r="E12" s="2" t="n">
-        <v>-27.5342</v>
-      </c>
-      <c r="F12" s="2" t="n">
-        <v>0.038</v>
-      </c>
-      <c r="G12" s="2" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>671705.4195</v>
-      </c>
-      <c r="D13" s="2" t="n">
-        <v>1507395.991</v>
-      </c>
-      <c r="E13" s="2" t="n">
-        <v>-27.9994</v>
-      </c>
-      <c r="F13" s="2" t="n">
-        <v>0.038</v>
-      </c>
-      <c r="G13" s="2" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>671703.7396</v>
-      </c>
-      <c r="D14" s="2" t="n">
-        <v>1507397.789</v>
-      </c>
-      <c r="E14" s="2" t="n">
-        <v>-27.9921</v>
-      </c>
-      <c r="F14" s="2" t="n">
-        <v>0.038</v>
-      </c>
-      <c r="G14" s="2" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="C15" s="2" t="n">
-        <v>671703.5187</v>
-      </c>
-      <c r="D15" s="2" t="n">
-        <v>1507398.033</v>
-      </c>
-      <c r="E15" s="2" t="n">
-        <v>-27.436</v>
-      </c>
-      <c r="F15" s="2" t="n">
-        <v>0.038</v>
-      </c>
-      <c r="G15" s="2" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="C16" s="2" t="n">
-        <v>671703.4754999999</v>
-      </c>
-      <c r="D16" s="2" t="n">
-        <v>1507398.085</v>
-      </c>
-      <c r="E16" s="2" t="n">
-        <v>-26.6546</v>
-      </c>
-      <c r="F16" s="2" t="n">
-        <v>0.038</v>
-      </c>
-      <c r="G16" s="2" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="C17" s="2" t="n">
+      <c r="B17" s="5" t="n">
         <v>671703.6907</v>
       </c>
-      <c r="D17" s="2" t="n">
+      <c r="C17" s="5" t="n">
         <v>1507397.861</v>
       </c>
-      <c r="E17" s="2" t="n">
+      <c r="D17" s="5" t="n">
         <v>-25.9127</v>
       </c>
-      <c r="F17" s="2" t="n">
-        <v>0.038</v>
-      </c>
-      <c r="G17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B18" s="2" t="n">
-        <v>1</v>
+        <v>671706.4312</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>671706.4312</v>
+        <v>1507396.634</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>1507396.634</v>
-      </c>
-      <c r="E18" s="2" t="n">
         <v>-26.0231</v>
-      </c>
-      <c r="F18" s="2" t="n">
-        <v>0.038</v>
-      </c>
-      <c r="G18" s="3" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="19">
@@ -880,147 +778,98 @@
         <v>2</v>
       </c>
       <c r="B19" s="2" t="n">
-        <v>2</v>
+        <v>671706.5934</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>671706.5934</v>
+        <v>1507396.453</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>1507396.453</v>
-      </c>
-      <c r="E19" s="2" t="n">
         <v>-26.7388</v>
       </c>
-      <c r="F19" s="2" t="n">
-        <v>0.038</v>
-      </c>
-      <c r="G19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B20" s="2" t="n">
-        <v>3</v>
+        <v>671706.5089</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>671706.5089</v>
+        <v>1507396.546</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>1507396.546</v>
-      </c>
-      <c r="E20" s="2" t="n">
         <v>-27.5219</v>
       </c>
-      <c r="F20" s="2" t="n">
-        <v>0.038</v>
-      </c>
-      <c r="G20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B21" s="2" t="n">
-        <v>4</v>
+        <v>671706.2911</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>671706.2911</v>
+        <v>1507396.77</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>1507396.77</v>
-      </c>
-      <c r="E21" s="2" t="n">
         <v>-27.9887</v>
       </c>
-      <c r="F21" s="2" t="n">
-        <v>0.038</v>
-      </c>
-      <c r="G21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B22" s="2" t="n">
-        <v>5</v>
+        <v>671704.6112</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>671704.6112</v>
+        <v>1507398.568</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>1507398.568</v>
-      </c>
-      <c r="E22" s="2" t="n">
         <v>-27.9804</v>
       </c>
-      <c r="F22" s="2" t="n">
-        <v>0.038</v>
-      </c>
-      <c r="G22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B23" s="2" t="n">
-        <v>6</v>
+        <v>671704.3903</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>671704.3903</v>
+        <v>1507398.812</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>1507398.812</v>
-      </c>
-      <c r="E23" s="2" t="n">
         <v>-27.4215</v>
       </c>
-      <c r="F23" s="2" t="n">
-        <v>0.038</v>
-      </c>
-      <c r="G23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="B24" s="2" t="n">
-        <v>7</v>
+        <v>671704.3471</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>671704.3471</v>
+        <v>1507398.864</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>1507398.864</v>
-      </c>
-      <c r="E24" s="2" t="n">
         <v>-26.6401</v>
       </c>
-      <c r="F24" s="2" t="n">
-        <v>0.038</v>
-      </c>
-      <c r="G24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="B25" s="2" t="n">
-        <v>8</v>
+        <v>671704.5623</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>671704.5623</v>
+        <v>1507398.64</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>1507398.64</v>
-      </c>
-      <c r="E25" s="2" t="n">
         <v>-25.9012</v>
       </c>
-      <c r="F25" s="2" t="n">
-        <v>0.038</v>
-      </c>
-      <c r="G25" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1036,377 +885,377 @@
   <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>POINT NO.</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>CHAINAGE</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>EASTING (M.)</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>NORTHING (M.)</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>ELEVATION (M.)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B2" s="7" t="n">
         <v>9842</v>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" s="7" t="n">
         <v>671699.1936999999</v>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" s="7" t="n">
         <v>1507392.45</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" s="7" t="n">
         <v>-26.9</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B3" s="7" t="n">
         <v>9842.5</v>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="C3" s="7" t="n">
         <v>671699.5572</v>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D3" s="7" t="n">
         <v>1507392.814</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" s="7" t="n">
         <v>-26.9</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" s="7" t="n">
         <v>9843</v>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" s="7" t="n">
         <v>671699.9208</v>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D4" s="7" t="n">
         <v>1507393.177</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="7" t="n">
         <v>-26.9</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" s="7" t="n">
         <v>9843.5</v>
       </c>
-      <c r="C5" s="2" t="n">
+      <c r="C5" s="7" t="n">
         <v>671700.2843000001</v>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D5" s="7" t="n">
         <v>1507393.541</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="7" t="n">
         <v>-26.9</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="n">
+      <c r="B6" s="7" t="n">
         <v>9844</v>
       </c>
-      <c r="C6" s="2" t="n">
+      <c r="C6" s="7" t="n">
         <v>671700.6478</v>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D6" s="7" t="n">
         <v>1507393.904</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="7" t="n">
         <v>-26.9</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B7" s="7" t="n">
         <v>9844.5</v>
       </c>
-      <c r="C7" s="2" t="n">
+      <c r="C7" s="7" t="n">
         <v>671701.0113</v>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D7" s="7" t="n">
         <v>1507394.268</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="7" t="n">
         <v>-26.9</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B8" s="7" t="n">
         <v>9845</v>
       </c>
-      <c r="C8" s="2" t="n">
+      <c r="C8" s="7" t="n">
         <v>671701.3748</v>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D8" s="7" t="n">
         <v>1507394.631</v>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="7" t="n">
         <v>-26.9</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B9" s="7" t="n">
         <v>9845.5</v>
       </c>
-      <c r="C9" s="2" t="n">
+      <c r="C9" s="7" t="n">
         <v>671701.7383</v>
       </c>
-      <c r="D9" s="2" t="n">
+      <c r="D9" s="7" t="n">
         <v>1507394.995</v>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="7" t="n">
         <v>-26.9</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B10" s="7" t="n">
         <v>9846</v>
       </c>
-      <c r="C10" s="2" t="n">
+      <c r="C10" s="7" t="n">
         <v>671702.1019</v>
       </c>
-      <c r="D10" s="2" t="n">
+      <c r="D10" s="7" t="n">
         <v>1507395.358</v>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" s="7" t="n">
         <v>-26.9</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="B11" s="7" t="n">
         <v>9846.5</v>
       </c>
-      <c r="C11" s="2" t="n">
+      <c r="C11" s="7" t="n">
         <v>671702.4654</v>
       </c>
-      <c r="D11" s="2" t="n">
+      <c r="D11" s="7" t="n">
         <v>1507395.722</v>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="E11" s="7" t="n">
         <v>-26.9</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="7" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="n">
+      <c r="B12" s="7" t="n">
         <v>9847</v>
       </c>
-      <c r="C12" s="2" t="n">
+      <c r="C12" s="7" t="n">
         <v>671702.8289</v>
       </c>
-      <c r="D12" s="2" t="n">
+      <c r="D12" s="7" t="n">
         <v>1507396.085</v>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="E12" s="7" t="n">
         <v>-26.9</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="2" t="n">
+      <c r="B13" s="7" t="n">
         <v>9847.5</v>
       </c>
-      <c r="C13" s="2" t="n">
+      <c r="C13" s="7" t="n">
         <v>671703.1924000001</v>
       </c>
-      <c r="D13" s="2" t="n">
+      <c r="D13" s="7" t="n">
         <v>1507396.449</v>
       </c>
-      <c r="E13" s="2" t="n">
+      <c r="E13" s="7" t="n">
         <v>-26.9</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="7" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="2" t="n">
+      <c r="B14" s="7" t="n">
         <v>9848</v>
       </c>
-      <c r="C14" s="2" t="n">
+      <c r="C14" s="7" t="n">
         <v>671703.556</v>
       </c>
-      <c r="D14" s="2" t="n">
+      <c r="D14" s="7" t="n">
         <v>1507396.812</v>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="E14" s="7" t="n">
         <v>-26.9</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
+      <c r="A15" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="2" t="n">
+      <c r="B15" s="7" t="n">
         <v>9848.5</v>
       </c>
-      <c r="C15" s="2" t="n">
+      <c r="C15" s="7" t="n">
         <v>671703.9195</v>
       </c>
-      <c r="D15" s="2" t="n">
+      <c r="D15" s="7" t="n">
         <v>1507397.176</v>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="E15" s="7" t="n">
         <v>-26.9</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="2" t="n">
+      <c r="B16" s="7" t="n">
         <v>9849</v>
       </c>
-      <c r="C16" s="2" t="n">
+      <c r="C16" s="7" t="n">
         <v>671704.2830000001</v>
       </c>
-      <c r="D16" s="2" t="n">
+      <c r="D16" s="7" t="n">
         <v>1507397.539</v>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="E16" s="7" t="n">
         <v>-26.9</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
+      <c r="A17" s="7" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="2" t="n">
+      <c r="B17" s="7" t="n">
         <v>9849.5</v>
       </c>
-      <c r="C17" s="2" t="n">
+      <c r="C17" s="7" t="n">
         <v>671704.6465</v>
       </c>
-      <c r="D17" s="2" t="n">
+      <c r="D17" s="7" t="n">
         <v>1507397.903</v>
       </c>
-      <c r="E17" s="2" t="n">
+      <c r="E17" s="7" t="n">
         <v>-26.9</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
+      <c r="A18" s="7" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="2" t="n">
+      <c r="B18" s="7" t="n">
         <v>9850</v>
       </c>
-      <c r="C18" s="2" t="n">
+      <c r="C18" s="7" t="n">
         <v>671705.01</v>
       </c>
-      <c r="D18" s="2" t="n">
+      <c r="D18" s="7" t="n">
         <v>1507398.266</v>
       </c>
-      <c r="E18" s="2" t="n">
+      <c r="E18" s="7" t="n">
         <v>-26.9</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
+      <c r="A19" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="2" t="n">
+      <c r="B19" s="7" t="n">
         <v>9850.5</v>
       </c>
-      <c r="C19" s="2" t="n">
+      <c r="C19" s="7" t="n">
         <v>671705.3735</v>
       </c>
-      <c r="D19" s="2" t="n">
+      <c r="D19" s="7" t="n">
         <v>1507398.63</v>
       </c>
-      <c r="E19" s="2" t="n">
+      <c r="E19" s="7" t="n">
         <v>-26.9</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="7" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="2" t="n">
+      <c r="B20" s="7" t="n">
         <v>9851</v>
       </c>
-      <c r="C20" s="2" t="n">
+      <c r="C20" s="7" t="n">
         <v>671705.737</v>
       </c>
-      <c r="D20" s="2" t="n">
+      <c r="D20" s="7" t="n">
         <v>1507398.993</v>
       </c>
-      <c r="E20" s="2" t="n">
+      <c r="E20" s="7" t="n">
         <v>-26.9</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
+      <c r="A21" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="2" t="n">
+      <c r="B21" s="7" t="n">
         <v>9851.5</v>
       </c>
-      <c r="C21" s="2" t="n">
+      <c r="C21" s="7" t="n">
         <v>671706.1004999999</v>
       </c>
-      <c r="D21" s="2" t="n">
+      <c r="D21" s="7" t="n">
         <v>1507399.357</v>
       </c>
-      <c r="E21" s="2" t="n">
+      <c r="E21" s="7" t="n">
         <v>-26.9</v>
       </c>
     </row>

</xml_diff>